<commit_message>
Finalize supporting Excel aligned with business exposure modelling
</commit_message>
<xml_diff>
--- a/Sprint1_Exposure_Calculator.xlsx
+++ b/Sprint1_Exposure_Calculator.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashok\Downloads\BTECH 3RD YEAR\6TH SEMESTER\BUSINESS ANALYTICS\Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashok\Downloads\BTECH 3RD YEAR\6TH SEMESTER\BUSINESS ANALYTICS\Project\FX-Decision-Recommendation-System-for-Indian-Businesses\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E00B5757-671F-4334-AA99-351FDA23F705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E987A12-8CFA-4C99-A003-B38A52BE4F38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{B9056E23-9CEF-48F6-AD93-70AE04465FF8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{B9056E23-9CEF-48F6-AD93-70AE04465FF8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Personas" sheetId="1" r:id="rId1"/>
-    <sheet name="Target_Rate_Impact" sheetId="2" r:id="rId2"/>
-    <sheet name="Exposure_Profiles" sheetId="3" r:id="rId3"/>
-    <sheet name="Break_Even_Rate" sheetId="4" r:id="rId4"/>
+    <sheet name="Assumptions" sheetId="1" r:id="rId1"/>
+    <sheet name="Scenario_Exposure" sheetId="2" r:id="rId2"/>
+    <sheet name="PaR_Thresholds" sheetId="3" r:id="rId3"/>
+    <sheet name="Summary_for_Decision" sheetId="4" r:id="rId4"/>
     <sheet name="Sensitivity_Analysis" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -38,83 +38,20 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="31">
-  <si>
-    <t>Business Type</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="32">
   <si>
     <t>USD Amount</t>
   </si>
   <si>
-    <t>Type</t>
-  </si>
-  <si>
     <t>Importer</t>
   </si>
   <si>
-    <t>Payable</t>
-  </si>
-  <si>
     <t>Exporter</t>
   </si>
   <si>
-    <t>Receivable</t>
-  </si>
-  <si>
     <t>IT Firm</t>
   </si>
   <si>
-    <t>Revenue</t>
-  </si>
-  <si>
-    <t>Current Rate</t>
-  </si>
-  <si>
-    <t>Target Rate</t>
-  </si>
-  <si>
-    <t>1% Impact (₹)</t>
-  </si>
-  <si>
-    <t>5% Impact (₹)</t>
-  </si>
-  <si>
-    <t>calculated</t>
-  </si>
-  <si>
-    <t>Current USD–INR = 83</t>
-  </si>
-  <si>
-    <t>Assume</t>
-  </si>
-  <si>
-    <t>Exposure Formula</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>USD × Rate Increase</t>
-  </si>
-  <si>
-    <t>Loss if INR weakens</t>
-  </si>
-  <si>
-    <t>USD × Rate Decrease</t>
-  </si>
-  <si>
-    <t>Loss if INR strengthens</t>
-  </si>
-  <si>
-    <t>(USD×Rate) − Costs</t>
-  </si>
-  <si>
-    <t>Profit sensitivity</t>
-  </si>
-  <si>
-    <t>INR Cost / Revenue</t>
-  </si>
-  <si>
     <t>Break-even Rate</t>
   </si>
   <si>
@@ -131,6 +68,73 @@
   </si>
   <si>
     <t>calc</t>
+  </si>
+  <si>
+    <t>Parameter</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Base USD–INR Rate</t>
+  </si>
+  <si>
+    <t>IT Firm INR Costs</t>
+  </si>
+  <si>
+    <t>Scenario</t>
+  </si>
+  <si>
+    <t>USD–INR Rate</t>
+  </si>
+  <si>
+    <t>Importer Impact (₹)</t>
+  </si>
+  <si>
+    <t>Exporter Impact (₹)</t>
+  </si>
+  <si>
+    <t>IT Firm Profit (₹)</t>
+  </si>
+  <si>
+    <t>Favorable</t>
+  </si>
+  <si>
+    <t>Neutral</t>
+  </si>
+  <si>
+    <t>Adverse</t>
+  </si>
+  <si>
+    <t>Business</t>
+  </si>
+  <si>
+    <t>Pain Threshold Rate</t>
+  </si>
+  <si>
+    <t>This spreadsheet provides a summarized view of business exposure analysis.
+Detailed scenario modelling, risk prioritisation, and exposure zoning are implemented in the Python notebook.</t>
+  </si>
+  <si>
+    <t>Risk Sensitivity</t>
+  </si>
+  <si>
+    <t>Key Risk Driver</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>INR depreciation increases costs</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Risk depends on direction</t>
+  </si>
+  <si>
+    <t>Margin sensitivity to FX</t>
   </si>
 </sst>
 </file>
@@ -499,55 +503,48 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
     <col min="3" max="3" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
       </c>
       <c r="B2" s="2">
         <v>10000</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>4</v>
-      </c>
+      <c r="C2" s="2"/>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2">
-        <v>10000</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>6</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="C3" s="2"/>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B4" s="2">
-        <v>10000</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>8</v>
-      </c>
+        <v>600000</v>
+      </c>
+      <c r="C4" s="2"/>
       <c r="D4" s="2"/>
     </row>
   </sheetData>
@@ -557,7 +554,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2CE86B9-6288-481F-9416-D295851D4123}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.5703125" customWidth="1"/>
@@ -567,97 +564,78 @@
   <sheetData>
     <row r="1" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="B2" s="2">
+        <v>82</v>
+      </c>
+      <c r="C2" s="2">
+        <v>-10000</v>
+      </c>
+      <c r="D2" s="2">
         <v>10000</v>
       </c>
-      <c r="C2" s="2">
-        <v>83</v>
-      </c>
-      <c r="D2" s="2">
-        <v>84</v>
-      </c>
       <c r="E2" s="2">
-        <f>10000*0.83</f>
-        <v>8300</v>
-      </c>
-      <c r="F2" s="2">
-        <f>10000*4.15</f>
-        <v>41500</v>
-      </c>
+        <v>220000</v>
+      </c>
+      <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B3" s="2">
-        <v>10000</v>
+        <v>83</v>
       </c>
       <c r="C3" s="2">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="D3" s="2">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="E3" s="2">
-        <f>10000*0.83</f>
-        <v>8300</v>
-      </c>
-      <c r="F3" s="2">
-        <f>10000*4.15</f>
-        <v>41500</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>230000</v>
+      </c>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B4" s="2">
-        <v>10000</v>
+        <v>85</v>
       </c>
       <c r="C4" s="2">
-        <v>83</v>
+        <v>20000</v>
       </c>
       <c r="D4" s="2">
-        <v>83</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>13</v>
-      </c>
+        <v>-20000</v>
+      </c>
+      <c r="E4" s="2">
+        <v>250000</v>
+      </c>
+      <c r="F4" s="2"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
+      <c r="A7" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -673,48 +651,48 @@
     <col min="3" max="3" width="19.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <v>83</v>
+      </c>
+      <c r="C2" s="2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>83</v>
+      </c>
+      <c r="C3" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>23</v>
+      <c r="B4" s="2">
+        <v>83</v>
+      </c>
+      <c r="C4" s="2">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -724,66 +702,67 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18D81048-F937-42FC-B87F-A9DE9B35EEB5}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="64.140625" customWidth="1"/>
+    <col min="2" max="2" width="12.85546875" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2">
-        <v>10000</v>
-      </c>
-      <c r="C2" s="2">
-        <v>850000</v>
-      </c>
-      <c r="D2" s="2">
-        <f>850000/10000</f>
-        <v>85</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="2">
-        <v>10000</v>
-      </c>
-      <c r="C3" s="2">
-        <v>750000</v>
-      </c>
-      <c r="D3" s="2">
-        <f>750000/10000</f>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="2">
-        <v>10000</v>
-      </c>
-      <c r="C4" s="2">
-        <v>600000</v>
-      </c>
-      <c r="D4" s="2">
-        <f>600000/10000</f>
-        <v>60</v>
+      <c r="B5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -798,16 +777,16 @@
   <sheetData>
     <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -821,7 +800,7 @@
         <v>5000</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -835,7 +814,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -849,7 +828,7 @@
         <v>-5000</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>